<commit_message>
Fixed global pair bug
</commit_message>
<xml_diff>
--- a/20240304_ternary_test copy/output/20240304_ternary_test copy_pairs.xlsx
+++ b/20240304_ternary_test copy/output/20240304_ternary_test copy_pairs.xlsx
@@ -1,26 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ge-Ge" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ge-Rh" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ge-Ru" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ge-Pr" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Eu-Ge" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ce-Ge" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ge-La" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ge-Ho" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ge-Sm" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ge-Nd" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ge-Ir" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ni-Ni" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ge-Ni" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ce-Ni" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="Ge-Ge" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Ge-Rh" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Ge-Ru" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Ge-Pr" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Eu-Ge" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Ce-Ge" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Ge-La" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Ge-Ho" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Ge-Sm" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Ge-Nd" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="Ge-Ir" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="Ni-Ni" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="Ge-Ni" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="Ce-Ni" sheetId="14" state="visible" r:id="rId14"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>

<commit_message>
Support order based on Mendeleev
</commit_message>
<xml_diff>
--- a/20240304_ternary_test copy/output/20240304_ternary_test copy_pairs.xlsx
+++ b/20240304_ternary_test copy/output/20240304_ternary_test copy_pairs.xlsx
@@ -8,19 +8,19 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ge-Ge" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ge-Rh" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ge-Ru" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ge-Pr" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rh-Ge" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ru-Ge" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pr-Ge" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Eu-Ge" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ce-Ge" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ge-La" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ge-Ho" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ge-Sm" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ge-Nd" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ge-Ir" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ge-Ni" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ni-Ni" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ce-Ni" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="La-Ge" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ho-Ge" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sm-Ge" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Nd-Ge" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ir-Ge" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ni-Ge" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ce-Ni" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ni-Ni" sheetId="14" state="visible" r:id="rId14"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -799,7 +799,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>2.226</v>
+        <v>3.141</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -845,7 +845,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>3.141</v>
+        <v>2.226</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Implement excel and json
</commit_message>
<xml_diff>
--- a/20240304_ternary_test copy/output/20240304_ternary_test copy_pairs.xlsx
+++ b/20240304_ternary_test copy/output/20240304_ternary_test copy_pairs.xlsx
@@ -1,14 +1,54 @@
+
+<file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <workbookPr/>
+  <workbookProtection/>
+  <bookViews>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+  </bookViews>
+  <sheets>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ru1-Ge1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="La1-Ge1" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ge1-Ge1" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ge,Ni1-Ge,Ni2" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pr-Ge,Ni2" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ge,Ni2-Ge,Ni2" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ge,Ni1-Ge,Ni1" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pr-Ge,Ni1" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pr1-Ge1" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rh1-Ge1" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ho1-Ge1" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sm1-Ge1" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Nd1-Ge1" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ir1-Ge1" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Eu1-Ge1" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ge1A-Ge1A" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ni1-Ge1A" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ni1-Ni1B" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ni1B-Ge1A" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ce1-Ge1A" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ni1B-Ni1B" sheetId="21" state="visible" r:id="rId21"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ce1-Ni1B" sheetId="22" state="visible" r:id="rId22"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ce1-Ge1" sheetId="23" state="visible" r:id="rId23"/>
+  </sheets>
+  <definedNames/>
+  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+</workbook>
+</file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -19,7 +59,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -27,12 +67,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -390,4 +439,1224 @@
   <a:objectDefaults/>
   <a:extraClrSchemeLst/>
 </a:theme>
+</file>
+
+<file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>File</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Mixing</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Distance</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>300168.cif</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>4</v>
+      </c>
+      <c r="C2" t="n">
+        <v>2.535</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>300170.cif</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>4</v>
+      </c>
+      <c r="C3" t="n">
+        <v>2.543</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>300169.cif</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>4</v>
+      </c>
+      <c r="C4" t="n">
+        <v>2.554</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>File</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Mixing</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Distance</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>300156.cif</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>4</v>
+      </c>
+      <c r="C2" t="n">
+        <v>2.481</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>300160.cif</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>4</v>
+      </c>
+      <c r="C3" t="n">
+        <v>2.499</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>300161.cif</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>4</v>
+      </c>
+      <c r="C4" t="n">
+        <v>2.515</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>300162.cif</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>4</v>
+      </c>
+      <c r="C5" t="n">
+        <v>2.519</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>300159.cif</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>4</v>
+      </c>
+      <c r="C6" t="n">
+        <v>2.538</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>File</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Mixing</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Distance</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>300156.cif</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>4</v>
+      </c>
+      <c r="C2" t="n">
+        <v>3.12</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>File</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Mixing</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Distance</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>300160.cif</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>4</v>
+      </c>
+      <c r="C2" t="n">
+        <v>3.141</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>File</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Mixing</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Distance</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>300161.cif</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>4</v>
+      </c>
+      <c r="C2" t="n">
+        <v>3.157</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>File</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Mixing</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Distance</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>300171.cif</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>4</v>
+      </c>
+      <c r="C2" t="n">
+        <v>2.537</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>File</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Mixing</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Distance</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>300159.cif</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>4</v>
+      </c>
+      <c r="C2" t="n">
+        <v>3.179</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>300171.cif</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>4</v>
+      </c>
+      <c r="C3" t="n">
+        <v>3.182</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>File</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Mixing</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Distance</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>1040392.cif</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>2</v>
+      </c>
+      <c r="C2" t="n">
+        <v>2.226</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>File</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Mixing</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Distance</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>1040392.cif</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>2</v>
+      </c>
+      <c r="C2" t="n">
+        <v>2.477</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>File</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Mixing</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Distance</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>1040392.cif</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>2</v>
+      </c>
+      <c r="C2" t="n">
+        <v>2.477</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>File</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Mixing</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Distance</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>1040392.cif</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>2</v>
+      </c>
+      <c r="C2" t="n">
+        <v>2.226</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>File</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Mixing</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Distance</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>300169.cif</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>4</v>
+      </c>
+      <c r="C2" t="n">
+        <v>3.241</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>File</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Mixing</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Distance</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>1040392.cif</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C2" t="n">
+        <v>3.141</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>File</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Mixing</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Distance</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>1040392.cif</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>2</v>
+      </c>
+      <c r="C2" t="n">
+        <v>2.226</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>File</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Mixing</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Distance</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>1040392.cif</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C2" t="n">
+        <v>3.141</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>File</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Mixing</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Distance</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>300170.cif</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>4</v>
+      </c>
+      <c r="C2" t="n">
+        <v>3.227</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C10"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>File</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Mixing</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Distance</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>300168.cif</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>4</v>
+      </c>
+      <c r="C2" t="n">
+        <v>2.265</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>300170.cif</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>4</v>
+      </c>
+      <c r="C3" t="n">
+        <v>2.28</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>300169.cif</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>4</v>
+      </c>
+      <c r="C4" t="n">
+        <v>2.29</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>300156.cif</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>4</v>
+      </c>
+      <c r="C5" t="n">
+        <v>2.304</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>300160.cif</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>4</v>
+      </c>
+      <c r="C6" t="n">
+        <v>2.329</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>300161.cif</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>4</v>
+      </c>
+      <c r="C7" t="n">
+        <v>2.352</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>300162.cif</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>4</v>
+      </c>
+      <c r="C8" t="n">
+        <v>2.359</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>300171.cif</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>4</v>
+      </c>
+      <c r="C9" t="n">
+        <v>2.383</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>300159.cif</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>4</v>
+      </c>
+      <c r="C10" t="n">
+        <v>2.396</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>File</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Mixing</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Distance</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>1005628.cif</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C2" t="n">
+        <v>2.401</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>File</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Mixing</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Distance</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>1005628.cif</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C2" t="n">
+        <v>3.168</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>File</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Mixing</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Distance</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>1005628.cif</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C2" t="n">
+        <v>2.401</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>File</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Mixing</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Distance</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>1005628.cif</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C2" t="n">
+        <v>2.401</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>File</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Mixing</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Distance</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>1005628.cif</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C2" t="n">
+        <v>3.168</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>File</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Mixing</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Distance</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>300162.cif</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>4</v>
+      </c>
+      <c r="C2" t="n">
+        <v>3.161</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>300168.cif</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>4</v>
+      </c>
+      <c r="C3" t="n">
+        <v>3.22</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>